<commit_message>
Restore and rebrand ten public free downloads; targeted dry run [skip deploy]
</commit_message>
<xml_diff>
--- a/products-storage/00-free-bankrotstvo-proverka/02-reestr-priznakov-po-obektu.xlsx
+++ b/products-storage/00-free-bankrotstvo-proverka/02-reestr-priznakov-po-obektu.xlsx
@@ -1138,35 +1138,41 @@
         </is>
       </c>
     </row>
-    <row r="63">
+    <row r="63" ht="28" customHeight="1">
       <c r="A63" s="2" t="inlineStr">
         <is>
           <t>Переход к платному комплекту</t>
         </is>
       </c>
     </row>
-    <row r="64">
+    <row r="64" ht="36" customHeight="1">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>Комплект «Реестр требований кредиторов: как подрядчику заявить требование, сроки, переписка с управляющим» — 2 990 ₽.</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
+          <t>Комплект «Система защиты требований подрядчика при банкротстве генподрядчика» - 24 900 ₽.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="28" customHeight="1">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>https://marzhavbetone.ru/products/p9-bankrotstvo-genpodryadchika.html</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
+          <t>https://nastoronepodryadchika.ru/products/p9-bankrotstvo-genpodryadchika.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="28" customHeight="1">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>Комплект не заменяет юриста и не гарантирует выплату: он про то, чтобы вовремя оказаться в реестре и корректно переписываться с управляющим.</t>
+          <t>Вопросы по комплекту: nastoronepodryadchika@yandex.ru</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A63:K63"/>
+    <mergeCell ref="A64:K64"/>
+    <mergeCell ref="A65:K65"/>
+    <mergeCell ref="A66:K66"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>